<commit_message>
Fix: cache bust load_buoyancy to read new estimates
</commit_message>
<xml_diff>
--- a/buoyancy_estimates.xlsx
+++ b/buoyancy_estimates.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\AQ\Tax Bouyancy TPO\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\LENOVO\Downloads\Pakistan_Income_Tax_Slabs_app\macro_forecasting_II\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3DB0BBC1-FB59-469B-8FBD-C3E404220E74}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BA7018C2-B8F0-4975-8E45-068EED795E10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="9518" yWindow="0" windowWidth="9765" windowHeight="10162" firstSheet="1" activeTab="2" xr2:uid="{A220C3EB-FB50-4D70-8594-0EAD70902D49}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="10276" firstSheet="1" activeTab="3" xr2:uid="{A220C3EB-FB50-4D70-8594-0EAD70902D49}"/>
   </bookViews>
   <sheets>
     <sheet name="Dataset Tax &amp; Tax Base" sheetId="1" r:id="rId1"/>
@@ -1064,6 +1064,15 @@
     <xf numFmtId="0" fontId="12" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="1" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="4" borderId="1" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1076,12 +1085,6 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="1" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="14" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1117,9 +1120,6 @@
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="6">
@@ -3049,28 +3049,28 @@
       </c>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.45">
-      <c r="B5" s="80" t="s">
+      <c r="B5" s="83" t="s">
         <v>1</v>
       </c>
-      <c r="C5" s="84" t="s">
+      <c r="C5" s="81" t="s">
         <v>40</v>
       </c>
-      <c r="D5" s="84"/>
-      <c r="E5" s="84"/>
-      <c r="F5" s="84"/>
-      <c r="G5" s="84"/>
-      <c r="H5" s="84"/>
+      <c r="D5" s="81"/>
+      <c r="E5" s="81"/>
+      <c r="F5" s="81"/>
+      <c r="G5" s="81"/>
+      <c r="H5" s="81"/>
       <c r="I5" s="13"/>
-      <c r="J5" s="79" t="s">
+      <c r="J5" s="82" t="s">
         <v>41</v>
       </c>
-      <c r="K5" s="79"/>
-      <c r="L5" s="79"/>
-      <c r="M5" s="79"/>
-      <c r="N5" s="79"/>
+      <c r="K5" s="82"/>
+      <c r="L5" s="82"/>
+      <c r="M5" s="82"/>
+      <c r="N5" s="82"/>
     </row>
     <row r="6" spans="1:14" ht="28.5" x14ac:dyDescent="0.45">
-      <c r="B6" s="80"/>
+      <c r="B6" s="83"/>
       <c r="C6" s="12" t="s">
         <v>42</v>
       </c>
@@ -4456,20 +4456,20 @@
       <c r="N38" s="45"/>
     </row>
     <row r="39" spans="3:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="C39" s="81" t="s">
+      <c r="C39" s="84" t="s">
         <v>82</v>
       </c>
-      <c r="D39" s="81"/>
-      <c r="E39" s="82" t="s">
+      <c r="D39" s="84"/>
+      <c r="E39" s="85" t="s">
         <v>83</v>
       </c>
-      <c r="F39" s="82"/>
-      <c r="G39" s="82"/>
-      <c r="H39" s="81" t="s">
+      <c r="F39" s="85"/>
+      <c r="G39" s="85"/>
+      <c r="H39" s="84" t="s">
         <v>84</v>
       </c>
-      <c r="I39" s="81"/>
-      <c r="J39" s="81"/>
+      <c r="I39" s="84"/>
+      <c r="J39" s="84"/>
     </row>
     <row r="40" spans="3:14" ht="32.65" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C40" s="20" t="s">
@@ -4478,18 +4478,18 @@
       <c r="D40" s="18">
         <v>10.8</v>
       </c>
-      <c r="E40" s="83" t="s">
+      <c r="E40" s="80" t="s">
         <v>42</v>
       </c>
-      <c r="F40" s="83"/>
+      <c r="F40" s="80"/>
       <c r="G40" s="21">
         <f>C35</f>
         <v>1.2398208626955942</v>
       </c>
-      <c r="H40" s="83" t="s">
+      <c r="H40" s="80" t="s">
         <v>48</v>
       </c>
-      <c r="I40" s="83"/>
+      <c r="I40" s="80"/>
       <c r="J40" s="21">
         <f>D40*G40</f>
         <v>13.390065317112418</v>
@@ -4503,18 +4503,18 @@
       <c r="D41" s="18">
         <v>4.9000000000000004</v>
       </c>
-      <c r="E41" s="83" t="s">
+      <c r="E41" s="80" t="s">
         <v>50</v>
       </c>
-      <c r="F41" s="83"/>
+      <c r="F41" s="80"/>
       <c r="G41" s="21">
         <f>E35</f>
         <v>1.0253543553331874</v>
       </c>
-      <c r="H41" s="83" t="s">
+      <c r="H41" s="80" t="s">
         <v>51</v>
       </c>
-      <c r="I41" s="83"/>
+      <c r="I41" s="80"/>
       <c r="J41" s="21">
         <f>D41*G41</f>
         <v>5.0242363411326183</v>
@@ -4527,18 +4527,18 @@
       <c r="D42" s="23">
         <v>13.4</v>
       </c>
-      <c r="E42" s="83" t="s">
+      <c r="E42" s="80" t="s">
         <v>43</v>
       </c>
-      <c r="F42" s="83"/>
+      <c r="F42" s="80"/>
       <c r="G42" s="21">
         <f>D35</f>
         <v>1.0085245836607837</v>
       </c>
-      <c r="H42" s="83" t="s">
+      <c r="H42" s="80" t="s">
         <v>53</v>
       </c>
-      <c r="I42" s="83"/>
+      <c r="I42" s="80"/>
       <c r="J42" s="21">
         <f>D42*G42</f>
         <v>13.514229421054502</v>
@@ -4551,18 +4551,18 @@
       <c r="D43" s="18">
         <v>6.1</v>
       </c>
-      <c r="E43" s="83" t="s">
+      <c r="E43" s="80" t="s">
         <v>55</v>
       </c>
-      <c r="F43" s="83"/>
+      <c r="F43" s="80"/>
       <c r="G43" s="21">
         <f>G35</f>
         <v>1.0364462480401231</v>
       </c>
-      <c r="H43" s="83" t="s">
+      <c r="H43" s="80" t="s">
         <v>56</v>
       </c>
-      <c r="I43" s="83"/>
+      <c r="I43" s="80"/>
       <c r="J43" s="21">
         <f>D42*G43</f>
         <v>13.88837972373765</v>
@@ -4575,18 +4575,18 @@
       <c r="D44" s="18">
         <v>4</v>
       </c>
-      <c r="E44" s="83" t="s">
+      <c r="E44" s="80" t="s">
         <v>45</v>
       </c>
-      <c r="F44" s="83"/>
+      <c r="F44" s="80"/>
       <c r="G44" s="21">
         <f>F35</f>
         <v>0.87999719404728449</v>
       </c>
-      <c r="H44" s="83" t="s">
+      <c r="H44" s="80" t="s">
         <v>58</v>
       </c>
-      <c r="I44" s="83"/>
+      <c r="I44" s="80"/>
       <c r="J44" s="21">
         <f>D41*G44</f>
         <v>4.3119862508316942</v>
@@ -4601,6 +4601,11 @@
     </row>
   </sheetData>
   <mergeCells count="16">
+    <mergeCell ref="J5:N5"/>
+    <mergeCell ref="B5:B6"/>
+    <mergeCell ref="C39:D39"/>
+    <mergeCell ref="E39:G39"/>
+    <mergeCell ref="H39:J39"/>
     <mergeCell ref="E43:F43"/>
     <mergeCell ref="H43:I43"/>
     <mergeCell ref="E44:F44"/>
@@ -4612,11 +4617,6 @@
     <mergeCell ref="H41:I41"/>
     <mergeCell ref="E42:F42"/>
     <mergeCell ref="H42:I42"/>
-    <mergeCell ref="J5:N5"/>
-    <mergeCell ref="B5:B6"/>
-    <mergeCell ref="C39:D39"/>
-    <mergeCell ref="E39:G39"/>
-    <mergeCell ref="H39:J39"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -4841,7 +4841,7 @@
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A13"/>
-      <c r="E13" s="97"/>
+      <c r="E13" s="79"/>
       <c r="F13"/>
       <c r="G13"/>
       <c r="H13"/>
@@ -4882,7 +4882,7 @@
   <sheetPr>
     <tabColor rgb="FF0070C0"/>
   </sheetPr>
-  <dimension ref="A1:I28"/>
+  <dimension ref="A1:R28"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="2" max="2" width="29.86328125" customWidth="1"/>
@@ -4895,13 +4895,13 @@
     <col min="9" max="9" width="9.59765625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="18" x14ac:dyDescent="0.55000000000000004">
+    <row r="1" spans="1:18" ht="18" x14ac:dyDescent="0.55000000000000004">
       <c r="A1" s="49" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="5" spans="1:9" ht="26.25" x14ac:dyDescent="0.45">
-      <c r="B5" s="85" t="s">
+    <row r="5" spans="1:18" ht="26.25" x14ac:dyDescent="0.45">
+      <c r="B5" s="86" t="s">
         <v>74</v>
       </c>
       <c r="C5" s="33" t="s">
@@ -4926,33 +4926,31 @@
         <v>6</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.45">
-      <c r="B6" s="85"/>
+    <row r="6" spans="1:18" x14ac:dyDescent="0.45">
+      <c r="B6" s="86"/>
       <c r="C6" s="35">
-        <v>6902000</v>
+        <v>6755478</v>
       </c>
       <c r="D6" s="41">
-        <f>0.61*F6</f>
-        <v>2899330</v>
+        <v>2640955</v>
       </c>
       <c r="E6" s="35">
-        <f>F6*0.39</f>
-        <v>1853670</v>
+        <v>1688480</v>
       </c>
       <c r="F6" s="35">
-        <v>4753000</v>
+        <v>4329435</v>
       </c>
       <c r="G6" s="41">
-        <v>888000</v>
+        <v>839352</v>
       </c>
       <c r="H6" s="41">
-        <v>1588000</v>
+        <v>1309059</v>
       </c>
       <c r="I6" s="35">
-        <v>14131000</v>
-      </c>
-    </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.45">
+        <v>13233324</v>
+      </c>
+    </row>
+    <row r="7" spans="1:18" x14ac:dyDescent="0.45">
       <c r="B7" s="66"/>
       <c r="C7" s="67"/>
       <c r="D7" s="68"/>
@@ -4961,8 +4959,15 @@
       <c r="G7" s="68"/>
       <c r="H7" s="68"/>
       <c r="I7" s="67"/>
-    </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="L7" s="26"/>
+      <c r="M7" s="26"/>
+      <c r="N7" s="26"/>
+      <c r="O7" s="26"/>
+      <c r="P7" s="26"/>
+      <c r="Q7" s="26"/>
+      <c r="R7" s="26"/>
+    </row>
+    <row r="8" spans="1:18" x14ac:dyDescent="0.45">
       <c r="B8" s="10"/>
       <c r="C8" s="10"/>
       <c r="D8" s="10"/>
@@ -4974,7 +4979,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:18" x14ac:dyDescent="0.45">
       <c r="B9" s="47"/>
       <c r="C9" s="47" t="s">
         <v>42</v>
@@ -4998,106 +5003,106 @@
         <v>64</v>
       </c>
     </row>
-    <row r="10" spans="1:9" ht="31.9" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:18" ht="31.9" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B10" s="19" t="s">
         <v>70</v>
       </c>
       <c r="C10" s="6">
         <f>'Sensitivity Analysis'!C6/1000</f>
-        <v>6902</v>
+        <v>6755.4780000000001</v>
       </c>
       <c r="D10" s="7">
         <f>'Sensitivity Analysis'!E6/1000</f>
-        <v>1853.67</v>
+        <v>1688.48</v>
       </c>
       <c r="E10" s="7">
         <f>'Sensitivity Analysis'!D6/1000</f>
-        <v>2899.33</v>
+        <v>2640.9549999999999</v>
       </c>
       <c r="F10" s="7">
         <f>SUM(D10:E10)</f>
-        <v>4753</v>
+        <v>4329.4349999999995</v>
       </c>
       <c r="G10" s="6">
         <f>H6/1000</f>
-        <v>1588</v>
+        <v>1309.059</v>
       </c>
       <c r="H10" s="6">
         <f>G6/1000</f>
-        <v>888</v>
+        <v>839.35199999999998</v>
       </c>
       <c r="I10" s="6">
         <f>I6/1000</f>
-        <v>14131</v>
-      </c>
-    </row>
-    <row r="11" spans="1:9" ht="29.65" customHeight="1" x14ac:dyDescent="0.45">
+        <v>13233.324000000001</v>
+      </c>
+    </row>
+    <row r="11" spans="1:18" ht="29.65" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B11" s="19" t="s">
         <v>59</v>
       </c>
       <c r="C11" s="7">
         <f>C10*('Tax Buoyancy Estimates'!J40/100)</f>
-        <v>924.18230818709912</v>
+        <v>904.56291668315964</v>
       </c>
       <c r="D11" s="8">
         <f>D10*('Tax Buoyancy Estimates'!J41/100)</f>
-        <v>93.132761784673008</v>
+        <v>84.833225772756023</v>
       </c>
       <c r="E11" s="8">
         <f>E10*('Tax Buoyancy Estimates'!J42/100)</f>
-        <v>391.82210787345952</v>
+        <v>356.90471760680992</v>
       </c>
       <c r="F11" s="8">
         <f>SUM(D11:E11)</f>
-        <v>484.95486965813251</v>
+        <v>441.73794337956593</v>
       </c>
       <c r="G11" s="7">
         <f>G10*('Tax Buoyancy Estimates'!J43/100)</f>
-        <v>220.54747001295391</v>
+        <v>181.80708472776286</v>
       </c>
       <c r="H11" s="9">
         <f>H10*('Tax Buoyancy Estimates'!J44/100)</f>
-        <v>38.290437907385439</v>
+        <v>36.192742836080839</v>
       </c>
       <c r="I11" s="8">
         <f>SUM(C11,F11,G11,H11)</f>
-        <v>1667.9750857655711</v>
-      </c>
-    </row>
-    <row r="12" spans="1:9" ht="34.5" customHeight="1" x14ac:dyDescent="0.45">
+        <v>1564.3006876265695</v>
+      </c>
+    </row>
+    <row r="12" spans="1:18" ht="34.5" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B12" s="19" t="s">
         <v>71</v>
       </c>
       <c r="C12" s="7">
         <f t="shared" ref="C12:H12" si="0">C10+C11</f>
-        <v>7826.1823081870989</v>
+        <v>7660.0409166831596</v>
       </c>
       <c r="D12" s="7">
         <f t="shared" si="0"/>
-        <v>1946.8027617846731</v>
+        <v>1773.3132257727561</v>
       </c>
       <c r="E12" s="7">
         <f t="shared" si="0"/>
-        <v>3291.1521078734595</v>
+        <v>2997.8597176068097</v>
       </c>
       <c r="F12" s="7">
         <f>F10+F11</f>
-        <v>5237.9548696581323</v>
+        <v>4771.1729433795654</v>
       </c>
       <c r="G12" s="7">
         <f t="shared" si="0"/>
-        <v>1808.5474700129539</v>
+        <v>1490.8660847277629</v>
       </c>
       <c r="H12" s="7">
         <f t="shared" si="0"/>
-        <v>926.29043790738547</v>
+        <v>875.54474283608079</v>
       </c>
       <c r="I12" s="7">
         <f>I10+I11</f>
-        <v>15798.975085765571</v>
-      </c>
-    </row>
-    <row r="13" spans="1:9" ht="28.5" x14ac:dyDescent="0.45">
+        <v>14797.62468762657</v>
+      </c>
+    </row>
+    <row r="13" spans="1:18" ht="28.5" x14ac:dyDescent="0.45">
       <c r="B13" s="19" t="s">
         <v>60</v>
       </c>
@@ -5130,7 +5135,7 @@
         <v>50.128897053868883</v>
       </c>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:18" x14ac:dyDescent="0.45">
       <c r="B14" s="10"/>
       <c r="C14" s="10"/>
       <c r="D14" s="10"/>
@@ -5140,7 +5145,7 @@
       <c r="H14" s="10"/>
       <c r="I14" s="10"/>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:18" x14ac:dyDescent="0.45">
       <c r="B15" s="10"/>
       <c r="C15" s="10"/>
       <c r="D15" s="10"/>
@@ -5150,7 +5155,7 @@
       <c r="H15" s="10"/>
       <c r="I15" s="10"/>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:18" x14ac:dyDescent="0.45">
       <c r="B16" s="10"/>
       <c r="C16" s="10"/>
       <c r="D16" s="10"/>
@@ -5214,31 +5219,31 @@
       </c>
       <c r="C20" s="7">
         <f t="shared" ref="C20:I20" si="1">C10</f>
-        <v>6902</v>
+        <v>6755.4780000000001</v>
       </c>
       <c r="D20" s="7">
         <f t="shared" si="1"/>
-        <v>1853.67</v>
+        <v>1688.48</v>
       </c>
       <c r="E20" s="7">
         <f t="shared" si="1"/>
-        <v>2899.33</v>
+        <v>2640.9549999999999</v>
       </c>
       <c r="F20" s="7">
         <f t="shared" si="1"/>
-        <v>4753</v>
+        <v>4329.4349999999995</v>
       </c>
       <c r="G20" s="7">
         <f t="shared" si="1"/>
-        <v>1588</v>
+        <v>1309.059</v>
       </c>
       <c r="H20" s="7">
         <f t="shared" si="1"/>
-        <v>888</v>
+        <v>839.35199999999998</v>
       </c>
       <c r="I20" s="7">
         <f t="shared" si="1"/>
-        <v>14131</v>
+        <v>13233.324000000001</v>
       </c>
     </row>
     <row r="21" spans="2:9" ht="29.25" customHeight="1" x14ac:dyDescent="0.45">
@@ -5280,25 +5285,25 @@
       </c>
       <c r="C22" s="7">
         <f>C20*(1+(C21/100))</f>
-        <v>7733.7640773683897</v>
+        <v>7569.5846250148443</v>
       </c>
       <c r="D22" s="7"/>
       <c r="E22" s="7"/>
       <c r="F22" s="7">
         <f>F20*(1+(F21/100))</f>
-        <v>5546.0199499090786</v>
+        <v>5051.7847426540311</v>
       </c>
       <c r="G22" s="7">
         <f>G20*(1+(G21/100))</f>
-        <v>1786.4927230116587</v>
+        <v>1472.6853762549867</v>
       </c>
       <c r="H22" s="7">
         <f>H20*(1+(H21/100))</f>
-        <v>922.46139411664694</v>
+        <v>871.92546855247281</v>
       </c>
       <c r="I22" s="7">
         <f>I20*(1+(I21/100))</f>
-        <v>20506.342998413991</v>
+        <v>19203.671428288431</v>
       </c>
     </row>
     <row r="23" spans="2:9" x14ac:dyDescent="0.45">
@@ -5353,31 +5358,31 @@
       </c>
       <c r="C26" s="7">
         <f t="shared" ref="C26:I26" si="3">C10</f>
-        <v>6902</v>
+        <v>6755.4780000000001</v>
       </c>
       <c r="D26" s="7">
         <f t="shared" si="3"/>
-        <v>1853.67</v>
+        <v>1688.48</v>
       </c>
       <c r="E26" s="7">
         <f t="shared" si="3"/>
-        <v>2899.33</v>
+        <v>2640.9549999999999</v>
       </c>
       <c r="F26" s="7">
         <f t="shared" si="3"/>
-        <v>4753</v>
+        <v>4329.4349999999995</v>
       </c>
       <c r="G26" s="7">
         <f t="shared" si="3"/>
-        <v>1588</v>
+        <v>1309.059</v>
       </c>
       <c r="H26" s="7">
         <f t="shared" si="3"/>
-        <v>888</v>
+        <v>839.35199999999998</v>
       </c>
       <c r="I26" s="7">
         <f t="shared" si="3"/>
-        <v>14131</v>
+        <v>13233.324000000001</v>
       </c>
     </row>
     <row r="27" spans="2:9" ht="33.75" customHeight="1" x14ac:dyDescent="0.45">
@@ -5419,25 +5424,25 @@
       </c>
       <c r="C28" s="7">
         <f>C26*(1+(C27/100))</f>
-        <v>7918.600539005809</v>
+        <v>7750.4972083514758</v>
       </c>
       <c r="D28" s="7"/>
       <c r="E28" s="7"/>
       <c r="F28" s="7">
         <f>F26*(1+(F27/100))</f>
-        <v>5722.2466054444294</v>
+        <v>5212.3069076882603</v>
       </c>
       <c r="G28" s="7">
         <f>G26*(1+(G27/100))</f>
-        <v>1830.6022170142492</v>
+        <v>1509.046793200539</v>
       </c>
       <c r="H28" s="7">
         <f>H26*(1+(H27/100))</f>
-        <v>930.1194816981241</v>
+        <v>879.16401711968899</v>
       </c>
       <c r="I28" s="7">
         <f>I26*(1+(I27/100))</f>
-        <v>21923.08588695043</v>
+        <v>20530.415301241417</v>
       </c>
     </row>
   </sheetData>
@@ -5461,7 +5466,7 @@
   <sheetData>
     <row r="1" spans="4:10" ht="14.65" thickBot="1" x14ac:dyDescent="0.5"/>
     <row r="2" spans="4:10" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="D2" s="89" t="s">
+      <c r="D2" s="90" t="s">
         <v>88</v>
       </c>
       <c r="E2" s="50" t="s">
@@ -5484,39 +5489,39 @@
       </c>
     </row>
     <row r="3" spans="4:10" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="D3" s="90"/>
+      <c r="D3" s="91"/>
       <c r="E3" s="53" t="s">
         <v>92</v>
       </c>
       <c r="F3" s="54" t="s">
         <v>93</v>
       </c>
-      <c r="G3" s="91" t="s">
+      <c r="G3" s="92" t="s">
         <v>94</v>
       </c>
-      <c r="H3" s="92"/>
-      <c r="I3" s="92"/>
-      <c r="J3" s="93"/>
+      <c r="H3" s="93"/>
+      <c r="I3" s="93"/>
+      <c r="J3" s="94"/>
     </row>
     <row r="4" spans="4:10" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="D4" s="94"/>
-      <c r="E4" s="95"/>
-      <c r="F4" s="95"/>
-      <c r="G4" s="95"/>
-      <c r="H4" s="95"/>
-      <c r="I4" s="95"/>
-      <c r="J4" s="96"/>
+      <c r="D4" s="95"/>
+      <c r="E4" s="96"/>
+      <c r="F4" s="96"/>
+      <c r="G4" s="96"/>
+      <c r="H4" s="96"/>
+      <c r="I4" s="96"/>
+      <c r="J4" s="97"/>
     </row>
     <row r="5" spans="4:10" ht="14.65" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="D5" s="86" t="s">
+      <c r="D5" s="87" t="s">
         <v>95</v>
       </c>
-      <c r="E5" s="87"/>
-      <c r="F5" s="87"/>
-      <c r="G5" s="87"/>
-      <c r="H5" s="87"/>
-      <c r="I5" s="87"/>
-      <c r="J5" s="88"/>
+      <c r="E5" s="88"/>
+      <c r="F5" s="88"/>
+      <c r="G5" s="88"/>
+      <c r="H5" s="88"/>
+      <c r="I5" s="88"/>
+      <c r="J5" s="89"/>
     </row>
     <row r="6" spans="4:10" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="D6" s="55" t="s">
@@ -5634,15 +5639,15 @@
       </c>
     </row>
     <row r="11" spans="4:10" ht="14.65" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="D11" s="86" t="s">
+      <c r="D11" s="87" t="s">
         <v>101</v>
       </c>
-      <c r="E11" s="87"/>
-      <c r="F11" s="87"/>
-      <c r="G11" s="87"/>
-      <c r="H11" s="87"/>
-      <c r="I11" s="87"/>
-      <c r="J11" s="88"/>
+      <c r="E11" s="88"/>
+      <c r="F11" s="88"/>
+      <c r="G11" s="88"/>
+      <c r="H11" s="88"/>
+      <c r="I11" s="88"/>
+      <c r="J11" s="89"/>
     </row>
     <row r="12" spans="4:10" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="D12" s="59" t="s">
@@ -5806,15 +5811,15 @@
       </c>
     </row>
     <row r="19" spans="4:10" ht="14.65" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="D19" s="86" t="s">
+      <c r="D19" s="87" t="s">
         <v>109</v>
       </c>
-      <c r="E19" s="87"/>
-      <c r="F19" s="87"/>
-      <c r="G19" s="87"/>
-      <c r="H19" s="87"/>
-      <c r="I19" s="87"/>
-      <c r="J19" s="88"/>
+      <c r="E19" s="88"/>
+      <c r="F19" s="88"/>
+      <c r="G19" s="88"/>
+      <c r="H19" s="88"/>
+      <c r="I19" s="88"/>
+      <c r="J19" s="89"/>
     </row>
     <row r="20" spans="4:10" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="D20" s="59" t="s">

</xml_diff>